<commit_message>
feat(cupmat): add UEFA Conference League fixtures with global team standards and i18n rules
</commit_message>
<xml_diff>
--- a/cupmat maç programı.xlsx
+++ b/cupmat maç programı.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026 dünya\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0624C81B-480C-49C3-8E00-378FD2529360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471C1C5F-77B1-4592-8C72-73574974D9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{41A974BD-A4C4-43BD-8942-2004F26BE2A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{41A974BD-A4C4-43BD-8942-2004F26BE2A2}"/>
   </bookViews>
   <sheets>
     <sheet name="U Şamp.L" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2001" uniqueCount="281">
   <si>
     <t>UEFA Şampiyonlar Ligi</t>
   </si>
@@ -626,6 +626,264 @@
   </si>
   <si>
     <t>UEFA Avrupa Ligi</t>
+  </si>
+  <si>
+    <t>Planet Group Arena</t>
+  </si>
+  <si>
+    <t>Gent</t>
+  </si>
+  <si>
+    <t>dk</t>
+  </si>
+  <si>
+    <t>AGF</t>
+  </si>
+  <si>
+    <t>AIL Arena</t>
+  </si>
+  <si>
+    <t>ch</t>
+  </si>
+  <si>
+    <t>Lugano</t>
+  </si>
+  <si>
+    <t>rs</t>
+  </si>
+  <si>
+    <t>Kızılyıldız</t>
+  </si>
+  <si>
+    <t>Gradski stadion u Poljudu</t>
+  </si>
+  <si>
+    <t>Hajduk Split</t>
+  </si>
+  <si>
+    <t>Ajax</t>
+  </si>
+  <si>
+    <t>Tammelan Stadion</t>
+  </si>
+  <si>
+    <t>fi</t>
+  </si>
+  <si>
+    <t>KuPS</t>
+  </si>
+  <si>
+    <t>Trabzonspor</t>
+  </si>
+  <si>
+    <t>ÇSKA Sofya</t>
+  </si>
+  <si>
+    <t>Monaco</t>
+  </si>
+  <si>
+    <t>Stadionul Ion Oblemenco</t>
+  </si>
+  <si>
+    <t>ro</t>
+  </si>
+  <si>
+    <t>CS U Craiova</t>
+  </si>
+  <si>
+    <t>Getafe</t>
+  </si>
+  <si>
+    <t>Olympiako Stadio Spyros Louis</t>
+  </si>
+  <si>
+    <t>Panathinaikos</t>
+  </si>
+  <si>
+    <t>ba</t>
+  </si>
+  <si>
+    <t>Borac Banja Luka</t>
+  </si>
+  <si>
+    <t>Olympia</t>
+  </si>
+  <si>
+    <t>se</t>
+  </si>
+  <si>
+    <t>Mjällby</t>
+  </si>
+  <si>
+    <t>ad</t>
+  </si>
+  <si>
+    <t>Inter Club</t>
+  </si>
+  <si>
+    <t>Stadions Skonto</t>
+  </si>
+  <si>
+    <t>lv</t>
+  </si>
+  <si>
+    <t>Riga FC</t>
+  </si>
+  <si>
+    <t>kz</t>
+  </si>
+  <si>
+    <t>Kairat</t>
+  </si>
+  <si>
+    <t>Elbasan Arena</t>
+  </si>
+  <si>
+    <t>al</t>
+  </si>
+  <si>
+    <t>Egnatia</t>
+  </si>
+  <si>
+    <t>Midtjylland</t>
+  </si>
+  <si>
+    <t>Europa-Park Stadion</t>
+  </si>
+  <si>
+    <t>Freiburg</t>
+  </si>
+  <si>
+    <t>Jablonec</t>
+  </si>
+  <si>
+    <t>Tynecastle Park</t>
+  </si>
+  <si>
+    <t>Hearts</t>
+  </si>
+  <si>
+    <t>Nordsjælland</t>
+  </si>
+  <si>
+    <t>Daio Wasabi Stayen Stadium</t>
+  </si>
+  <si>
+    <t>STVV</t>
+  </si>
+  <si>
+    <t>ge</t>
+  </si>
+  <si>
+    <t>Saburtalo</t>
+  </si>
+  <si>
+    <t>Brann Stadion</t>
+  </si>
+  <si>
+    <t>Brann</t>
+  </si>
+  <si>
+    <t>gi</t>
+  </si>
+  <si>
+    <t>Lincoln</t>
+  </si>
+  <si>
+    <t>Parken</t>
+  </si>
+  <si>
+    <t>Kopenhag</t>
+  </si>
+  <si>
+    <t>Braga</t>
+  </si>
+  <si>
+    <t>The American Express Stadium</t>
+  </si>
+  <si>
+    <t>Brighton</t>
+  </si>
+  <si>
+    <t>lt</t>
+  </si>
+  <si>
+    <t>Kauno Žalgiris</t>
+  </si>
+  <si>
+    <t>New Balance Arena</t>
+  </si>
+  <si>
+    <t>Atalanta</t>
+  </si>
+  <si>
+    <t>Pafos</t>
+  </si>
+  <si>
+    <t>De Grolsch Veste</t>
+  </si>
+  <si>
+    <t>Twente</t>
+  </si>
+  <si>
+    <t>Thun</t>
+  </si>
+  <si>
+    <t>Ortalıq Stadion</t>
+  </si>
+  <si>
+    <t>Coliseum Alfonso Pérez</t>
+  </si>
+  <si>
+    <t>Estadi de la FAF</t>
+  </si>
+  <si>
+    <t>Papara Park Stadyumu</t>
+  </si>
+  <si>
+    <t>Mikheil Meskhis Sakhelobis Stadioni</t>
+  </si>
+  <si>
+    <t>Right to Dream Park</t>
+  </si>
+  <si>
+    <t>Stadion Střelnice</t>
+  </si>
+  <si>
+    <t>S. Dariaus ir S. Girėno stadionas</t>
+  </si>
+  <si>
+    <t>Stadion Rajko Mitić</t>
+  </si>
+  <si>
+    <t>Alphamega Stadium</t>
+  </si>
+  <si>
+    <t>Cepheus Park Randers</t>
+  </si>
+  <si>
+    <t>Gradski Stadion</t>
+  </si>
+  <si>
+    <t>Stockhorn Arena</t>
+  </si>
+  <si>
+    <t>Europa Point Stadium</t>
+  </si>
+  <si>
+    <t>Johan Cruijff Arena</t>
+  </si>
+  <si>
+    <t>Stade Louis II</t>
+  </si>
+  <si>
+    <t>Estádio Municipal de Braga</t>
+  </si>
+  <si>
+    <t>MCH Arena</t>
+  </si>
+  <si>
+    <t>UEFA Konferans Ligi</t>
   </si>
 </sst>
 </file>
@@ -8665,9 +8923,2826 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D99B4F1-32AD-406C-BF6B-97E4F277565A}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:I109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:9" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="B1" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+    </row>
+    <row r="2" spans="2:9" ht="24" x14ac:dyDescent="0.4">
+      <c r="B2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G4" t="s">
+        <v>196</v>
+      </c>
+      <c r="H4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E5" t="s">
+        <v>199</v>
+      </c>
+      <c r="F5" t="s">
+        <v>200</v>
+      </c>
+      <c r="G5" t="s">
+        <v>201</v>
+      </c>
+      <c r="H5" t="s">
+        <v>202</v>
+      </c>
+      <c r="I5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E6" t="s">
+        <v>204</v>
+      </c>
+      <c r="F6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G6" t="s">
+        <v>205</v>
+      </c>
+      <c r="H6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E7" t="s">
+        <v>207</v>
+      </c>
+      <c r="F7" t="s">
+        <v>208</v>
+      </c>
+      <c r="G7" t="s">
+        <v>209</v>
+      </c>
+      <c r="H7" t="s">
+        <v>148</v>
+      </c>
+      <c r="I7" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" t="s">
+        <v>145</v>
+      </c>
+      <c r="G8" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" t="s">
+        <v>154</v>
+      </c>
+      <c r="I8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E9" t="s">
+        <v>213</v>
+      </c>
+      <c r="F9" t="s">
+        <v>214</v>
+      </c>
+      <c r="G9" t="s">
+        <v>215</v>
+      </c>
+      <c r="H9" t="s">
+        <v>150</v>
+      </c>
+      <c r="I9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E10" t="s">
+        <v>217</v>
+      </c>
+      <c r="F10" t="s">
+        <v>138</v>
+      </c>
+      <c r="G10" t="s">
+        <v>218</v>
+      </c>
+      <c r="H10" t="s">
+        <v>219</v>
+      </c>
+      <c r="I10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E11" t="s">
+        <v>221</v>
+      </c>
+      <c r="F11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G11" t="s">
+        <v>223</v>
+      </c>
+      <c r="H11" t="s">
+        <v>224</v>
+      </c>
+      <c r="I11" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F12" t="s">
+        <v>227</v>
+      </c>
+      <c r="G12" t="s">
+        <v>228</v>
+      </c>
+      <c r="H12" t="s">
+        <v>229</v>
+      </c>
+      <c r="I12" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E13" t="s">
+        <v>231</v>
+      </c>
+      <c r="F13" t="s">
+        <v>232</v>
+      </c>
+      <c r="G13" t="s">
+        <v>233</v>
+      </c>
+      <c r="H13" t="s">
+        <v>197</v>
+      </c>
+      <c r="I13" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E14" t="s">
+        <v>235</v>
+      </c>
+      <c r="F14" t="s">
+        <v>140</v>
+      </c>
+      <c r="G14" t="s">
+        <v>236</v>
+      </c>
+      <c r="H14" t="s">
+        <v>147</v>
+      </c>
+      <c r="I14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E15" t="s">
+        <v>238</v>
+      </c>
+      <c r="F15" t="s">
+        <v>146</v>
+      </c>
+      <c r="G15" t="s">
+        <v>239</v>
+      </c>
+      <c r="H15" t="s">
+        <v>197</v>
+      </c>
+      <c r="I15" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E16" t="s">
+        <v>241</v>
+      </c>
+      <c r="F16" t="s">
+        <v>139</v>
+      </c>
+      <c r="G16" t="s">
+        <v>242</v>
+      </c>
+      <c r="H16" t="s">
+        <v>243</v>
+      </c>
+      <c r="I16" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F17" t="s">
+        <v>149</v>
+      </c>
+      <c r="G17" t="s">
+        <v>246</v>
+      </c>
+      <c r="H17" t="s">
+        <v>247</v>
+      </c>
+      <c r="I17" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E18" t="s">
+        <v>249</v>
+      </c>
+      <c r="F18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G18" t="s">
+        <v>250</v>
+      </c>
+      <c r="H18" t="s">
+        <v>151</v>
+      </c>
+      <c r="I18" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E19" t="s">
+        <v>252</v>
+      </c>
+      <c r="F19" t="s">
+        <v>141</v>
+      </c>
+      <c r="G19" t="s">
+        <v>253</v>
+      </c>
+      <c r="H19" t="s">
+        <v>254</v>
+      </c>
+      <c r="I19" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E20" t="s">
+        <v>256</v>
+      </c>
+      <c r="F20" t="s">
+        <v>142</v>
+      </c>
+      <c r="G20" t="s">
+        <v>257</v>
+      </c>
+      <c r="H20" t="s">
+        <v>136</v>
+      </c>
+      <c r="I20" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E21" t="s">
+        <v>259</v>
+      </c>
+      <c r="F21" t="s">
+        <v>153</v>
+      </c>
+      <c r="G21" t="s">
+        <v>260</v>
+      </c>
+      <c r="H21" t="s">
+        <v>200</v>
+      </c>
+      <c r="I21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="E22" t="s">
+        <v>262</v>
+      </c>
+      <c r="F22" t="s">
+        <v>229</v>
+      </c>
+      <c r="G22" t="s">
+        <v>230</v>
+      </c>
+      <c r="H22" t="s">
+        <v>138</v>
+      </c>
+      <c r="I22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E23" t="s">
+        <v>263</v>
+      </c>
+      <c r="F23" t="s">
+        <v>150</v>
+      </c>
+      <c r="G23" t="s">
+        <v>216</v>
+      </c>
+      <c r="H23" t="s">
+        <v>200</v>
+      </c>
+      <c r="I23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>2</v>
+      </c>
+      <c r="C24" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E24" t="s">
+        <v>264</v>
+      </c>
+      <c r="F24" t="s">
+        <v>224</v>
+      </c>
+      <c r="G24" t="s">
+        <v>225</v>
+      </c>
+      <c r="H24" t="s">
+        <v>214</v>
+      </c>
+      <c r="I24" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E25" t="s">
+        <v>265</v>
+      </c>
+      <c r="F25" t="s">
+        <v>148</v>
+      </c>
+      <c r="G25" t="s">
+        <v>210</v>
+      </c>
+      <c r="H25" t="s">
+        <v>146</v>
+      </c>
+      <c r="I25" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E26" t="s">
+        <v>266</v>
+      </c>
+      <c r="F26" t="s">
+        <v>243</v>
+      </c>
+      <c r="G26" t="s">
+        <v>244</v>
+      </c>
+      <c r="H26" t="s">
+        <v>222</v>
+      </c>
+      <c r="I26" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E27" t="s">
+        <v>267</v>
+      </c>
+      <c r="F27" t="s">
+        <v>197</v>
+      </c>
+      <c r="G27" t="s">
+        <v>240</v>
+      </c>
+      <c r="H27" t="s">
+        <v>145</v>
+      </c>
+      <c r="I27" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E28" t="s">
+        <v>268</v>
+      </c>
+      <c r="F28" t="s">
+        <v>147</v>
+      </c>
+      <c r="G28" t="s">
+        <v>237</v>
+      </c>
+      <c r="H28" t="s">
+        <v>141</v>
+      </c>
+      <c r="I28" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E29" t="s">
+        <v>269</v>
+      </c>
+      <c r="F29" t="s">
+        <v>254</v>
+      </c>
+      <c r="G29" t="s">
+        <v>255</v>
+      </c>
+      <c r="H29" t="s">
+        <v>149</v>
+      </c>
+      <c r="I29" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E30" t="s">
+        <v>270</v>
+      </c>
+      <c r="F30" t="s">
+        <v>202</v>
+      </c>
+      <c r="G30" t="s">
+        <v>203</v>
+      </c>
+      <c r="H30" t="s">
+        <v>197</v>
+      </c>
+      <c r="I30" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>2</v>
+      </c>
+      <c r="C31" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E31" t="s">
+        <v>271</v>
+      </c>
+      <c r="F31" t="s">
+        <v>136</v>
+      </c>
+      <c r="G31" t="s">
+        <v>258</v>
+      </c>
+      <c r="H31" t="s">
+        <v>227</v>
+      </c>
+      <c r="I31" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>2</v>
+      </c>
+      <c r="C32" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E32" t="s">
+        <v>272</v>
+      </c>
+      <c r="F32" t="s">
+        <v>197</v>
+      </c>
+      <c r="G32" t="s">
+        <v>198</v>
+      </c>
+      <c r="H32" t="s">
+        <v>232</v>
+      </c>
+      <c r="I32" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E33" t="s">
+        <v>273</v>
+      </c>
+      <c r="F33" t="s">
+        <v>219</v>
+      </c>
+      <c r="G33" t="s">
+        <v>220</v>
+      </c>
+      <c r="H33" t="s">
+        <v>208</v>
+      </c>
+      <c r="I33" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E34" t="s">
+        <v>274</v>
+      </c>
+      <c r="F34" t="s">
+        <v>200</v>
+      </c>
+      <c r="G34" t="s">
+        <v>261</v>
+      </c>
+      <c r="H34" t="s">
+        <v>157</v>
+      </c>
+      <c r="I34" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E35" t="s">
+        <v>275</v>
+      </c>
+      <c r="F35" t="s">
+        <v>247</v>
+      </c>
+      <c r="G35" t="s">
+        <v>248</v>
+      </c>
+      <c r="H35" t="s">
+        <v>153</v>
+      </c>
+      <c r="I35" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D36" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E36" t="s">
+        <v>276</v>
+      </c>
+      <c r="F36" t="s">
+        <v>153</v>
+      </c>
+      <c r="G36" t="s">
+        <v>206</v>
+      </c>
+      <c r="H36" t="s">
+        <v>142</v>
+      </c>
+      <c r="I36" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E37" t="s">
+        <v>277</v>
+      </c>
+      <c r="F37" t="s">
+        <v>154</v>
+      </c>
+      <c r="G37" t="s">
+        <v>212</v>
+      </c>
+      <c r="H37" t="s">
+        <v>140</v>
+      </c>
+      <c r="I37" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>2</v>
+      </c>
+      <c r="C38" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D38" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E38" t="s">
+        <v>278</v>
+      </c>
+      <c r="F38" t="s">
+        <v>151</v>
+      </c>
+      <c r="G38" t="s">
+        <v>251</v>
+      </c>
+      <c r="H38" t="s">
+        <v>139</v>
+      </c>
+      <c r="I38" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D39" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E39" t="s">
+        <v>279</v>
+      </c>
+      <c r="F39" t="s">
+        <v>197</v>
+      </c>
+      <c r="G39" t="s">
+        <v>234</v>
+      </c>
+      <c r="H39" t="s">
+        <v>139</v>
+      </c>
+      <c r="I39" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D40" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E40" t="s">
+        <v>270</v>
+      </c>
+      <c r="F40" t="s">
+        <v>202</v>
+      </c>
+      <c r="G40" t="s">
+        <v>203</v>
+      </c>
+      <c r="H40" t="s">
+        <v>224</v>
+      </c>
+      <c r="I40" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41">
+        <v>3</v>
+      </c>
+      <c r="C41" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D41" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E41" t="s">
+        <v>265</v>
+      </c>
+      <c r="F41" t="s">
+        <v>148</v>
+      </c>
+      <c r="G41" t="s">
+        <v>210</v>
+      </c>
+      <c r="H41" t="s">
+        <v>140</v>
+      </c>
+      <c r="I41" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D42" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E42" t="s">
+        <v>275</v>
+      </c>
+      <c r="F42" t="s">
+        <v>247</v>
+      </c>
+      <c r="G42" t="s">
+        <v>248</v>
+      </c>
+      <c r="H42" t="s">
+        <v>157</v>
+      </c>
+      <c r="I42" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D43" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E43" t="s">
+        <v>207</v>
+      </c>
+      <c r="F43" t="s">
+        <v>208</v>
+      </c>
+      <c r="G43" t="s">
+        <v>209</v>
+      </c>
+      <c r="H43" t="s">
+        <v>139</v>
+      </c>
+      <c r="I43" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E44" t="s">
+        <v>279</v>
+      </c>
+      <c r="F44" t="s">
+        <v>197</v>
+      </c>
+      <c r="G44" t="s">
+        <v>234</v>
+      </c>
+      <c r="H44" t="s">
+        <v>153</v>
+      </c>
+      <c r="I44" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D45" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E45" t="s">
+        <v>272</v>
+      </c>
+      <c r="F45" t="s">
+        <v>197</v>
+      </c>
+      <c r="G45" t="s">
+        <v>198</v>
+      </c>
+      <c r="H45" t="s">
+        <v>151</v>
+      </c>
+      <c r="I45" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D46" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E46" t="s">
+        <v>274</v>
+      </c>
+      <c r="F46" t="s">
+        <v>200</v>
+      </c>
+      <c r="G46" t="s">
+        <v>261</v>
+      </c>
+      <c r="H46" t="s">
+        <v>146</v>
+      </c>
+      <c r="I46" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47">
+        <v>3</v>
+      </c>
+      <c r="C47" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D47" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E47" t="s">
+        <v>256</v>
+      </c>
+      <c r="F47" t="s">
+        <v>142</v>
+      </c>
+      <c r="G47" t="s">
+        <v>257</v>
+      </c>
+      <c r="H47" t="s">
+        <v>229</v>
+      </c>
+      <c r="I47" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48">
+        <v>3</v>
+      </c>
+      <c r="C48" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D48" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E48" t="s">
+        <v>221</v>
+      </c>
+      <c r="F48" t="s">
+        <v>222</v>
+      </c>
+      <c r="G48" t="s">
+        <v>223</v>
+      </c>
+      <c r="H48" t="s">
+        <v>219</v>
+      </c>
+      <c r="I48" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D49" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E49" t="s">
+        <v>213</v>
+      </c>
+      <c r="F49" t="s">
+        <v>214</v>
+      </c>
+      <c r="G49" t="s">
+        <v>215</v>
+      </c>
+      <c r="H49" t="s">
+        <v>232</v>
+      </c>
+      <c r="I49" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D50" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E50" t="s">
+        <v>259</v>
+      </c>
+      <c r="F50" t="s">
+        <v>153</v>
+      </c>
+      <c r="G50" t="s">
+        <v>260</v>
+      </c>
+      <c r="H50" t="s">
+        <v>136</v>
+      </c>
+      <c r="I50" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D51" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E51" t="s">
+        <v>263</v>
+      </c>
+      <c r="F51" t="s">
+        <v>150</v>
+      </c>
+      <c r="G51" t="s">
+        <v>216</v>
+      </c>
+      <c r="H51" t="s">
+        <v>141</v>
+      </c>
+      <c r="I51" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D52" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E52" t="s">
+        <v>217</v>
+      </c>
+      <c r="F52" t="s">
+        <v>138</v>
+      </c>
+      <c r="G52" t="s">
+        <v>218</v>
+      </c>
+      <c r="H52" t="s">
+        <v>145</v>
+      </c>
+      <c r="I52" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B53">
+        <v>3</v>
+      </c>
+      <c r="C53" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D53" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E53" t="s">
+        <v>226</v>
+      </c>
+      <c r="F53" t="s">
+        <v>227</v>
+      </c>
+      <c r="G53" t="s">
+        <v>228</v>
+      </c>
+      <c r="H53" t="s">
+        <v>147</v>
+      </c>
+      <c r="I53" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B54">
+        <v>3</v>
+      </c>
+      <c r="C54" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D54" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E54" t="s">
+        <v>249</v>
+      </c>
+      <c r="F54" t="s">
+        <v>197</v>
+      </c>
+      <c r="G54" t="s">
+        <v>250</v>
+      </c>
+      <c r="H54" t="s">
+        <v>243</v>
+      </c>
+      <c r="I54" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B55">
+        <v>3</v>
+      </c>
+      <c r="C55" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D55" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E55" t="s">
+        <v>199</v>
+      </c>
+      <c r="F55" t="s">
+        <v>200</v>
+      </c>
+      <c r="G55" t="s">
+        <v>201</v>
+      </c>
+      <c r="H55" t="s">
+        <v>254</v>
+      </c>
+      <c r="I55" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <v>3</v>
+      </c>
+      <c r="C56" s="2">
+        <v>46331</v>
+      </c>
+      <c r="D56" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E56" t="s">
+        <v>277</v>
+      </c>
+      <c r="F56" t="s">
+        <v>154</v>
+      </c>
+      <c r="G56" t="s">
+        <v>212</v>
+      </c>
+      <c r="H56" t="s">
+        <v>197</v>
+      </c>
+      <c r="I56" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="D57" s="3">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>241</v>
+      </c>
+      <c r="F57" t="s">
+        <v>139</v>
+      </c>
+      <c r="G57" t="s">
+        <v>242</v>
+      </c>
+      <c r="H57" t="s">
+        <v>149</v>
+      </c>
+      <c r="I57" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B58">
+        <v>4</v>
+      </c>
+      <c r="C58" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D58" s="3">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E58" t="s">
+        <v>262</v>
+      </c>
+      <c r="F58" t="s">
+        <v>229</v>
+      </c>
+      <c r="G58" t="s">
+        <v>230</v>
+      </c>
+      <c r="H58" t="s">
+        <v>222</v>
+      </c>
+      <c r="I58" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B59">
+        <v>4</v>
+      </c>
+      <c r="C59" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D59" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E59" t="s">
+        <v>245</v>
+      </c>
+      <c r="F59" t="s">
+        <v>149</v>
+      </c>
+      <c r="G59" t="s">
+        <v>246</v>
+      </c>
+      <c r="H59" t="s">
+        <v>197</v>
+      </c>
+      <c r="I59" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B60">
+        <v>4</v>
+      </c>
+      <c r="C60" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D60" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E60" t="s">
+        <v>271</v>
+      </c>
+      <c r="F60" t="s">
+        <v>136</v>
+      </c>
+      <c r="G60" t="s">
+        <v>258</v>
+      </c>
+      <c r="H60" t="s">
+        <v>197</v>
+      </c>
+      <c r="I60" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B61">
+        <v>4</v>
+      </c>
+      <c r="C61" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D61" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E61" t="s">
+        <v>252</v>
+      </c>
+      <c r="F61" t="s">
+        <v>141</v>
+      </c>
+      <c r="G61" t="s">
+        <v>253</v>
+      </c>
+      <c r="H61" t="s">
+        <v>214</v>
+      </c>
+      <c r="I61" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B62">
+        <v>4</v>
+      </c>
+      <c r="C62" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D62" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E62" t="s">
+        <v>268</v>
+      </c>
+      <c r="F62" t="s">
+        <v>147</v>
+      </c>
+      <c r="G62" t="s">
+        <v>237</v>
+      </c>
+      <c r="H62" t="s">
+        <v>200</v>
+      </c>
+      <c r="I62" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B63">
+        <v>4</v>
+      </c>
+      <c r="C63" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D63" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E63" t="s">
+        <v>269</v>
+      </c>
+      <c r="F63" t="s">
+        <v>254</v>
+      </c>
+      <c r="G63" t="s">
+        <v>255</v>
+      </c>
+      <c r="H63" t="s">
+        <v>227</v>
+      </c>
+      <c r="I63" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="64" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B64">
+        <v>4</v>
+      </c>
+      <c r="C64" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D64" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E64" t="s">
+        <v>276</v>
+      </c>
+      <c r="F64" t="s">
+        <v>153</v>
+      </c>
+      <c r="G64" t="s">
+        <v>206</v>
+      </c>
+      <c r="H64" t="s">
+        <v>200</v>
+      </c>
+      <c r="I64" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="65" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B65">
+        <v>4</v>
+      </c>
+      <c r="C65" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D65" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E65" t="s">
+        <v>231</v>
+      </c>
+      <c r="F65" t="s">
+        <v>232</v>
+      </c>
+      <c r="G65" t="s">
+        <v>233</v>
+      </c>
+      <c r="H65" t="s">
+        <v>247</v>
+      </c>
+      <c r="I65" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B66">
+        <v>4</v>
+      </c>
+      <c r="C66" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D66" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E66" t="s">
+        <v>238</v>
+      </c>
+      <c r="F66" t="s">
+        <v>146</v>
+      </c>
+      <c r="G66" t="s">
+        <v>239</v>
+      </c>
+      <c r="H66" t="s">
+        <v>154</v>
+      </c>
+      <c r="I66" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="67" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B67">
+        <v>4</v>
+      </c>
+      <c r="C67" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D67" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E67" t="s">
+        <v>266</v>
+      </c>
+      <c r="F67" t="s">
+        <v>243</v>
+      </c>
+      <c r="G67" t="s">
+        <v>244</v>
+      </c>
+      <c r="H67" t="s">
+        <v>150</v>
+      </c>
+      <c r="I67" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="68" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B68">
+        <v>4</v>
+      </c>
+      <c r="C68" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D68" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E68" t="s">
+        <v>235</v>
+      </c>
+      <c r="F68" t="s">
+        <v>140</v>
+      </c>
+      <c r="G68" t="s">
+        <v>236</v>
+      </c>
+      <c r="H68" t="s">
+        <v>153</v>
+      </c>
+      <c r="I68" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="69" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B69">
+        <v>4</v>
+      </c>
+      <c r="C69" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D69" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E69" t="s">
+        <v>267</v>
+      </c>
+      <c r="F69" t="s">
+        <v>197</v>
+      </c>
+      <c r="G69" t="s">
+        <v>240</v>
+      </c>
+      <c r="H69" t="s">
+        <v>138</v>
+      </c>
+      <c r="I69" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="70" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B70">
+        <v>4</v>
+      </c>
+      <c r="C70" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D70" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E70" t="s">
+        <v>264</v>
+      </c>
+      <c r="F70" t="s">
+        <v>224</v>
+      </c>
+      <c r="G70" t="s">
+        <v>225</v>
+      </c>
+      <c r="H70" t="s">
+        <v>197</v>
+      </c>
+      <c r="I70" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="71" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B71">
+        <v>4</v>
+      </c>
+      <c r="C71" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D71" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E71" t="s">
+        <v>107</v>
+      </c>
+      <c r="F71" t="s">
+        <v>145</v>
+      </c>
+      <c r="G71" t="s">
+        <v>211</v>
+      </c>
+      <c r="H71" t="s">
+        <v>148</v>
+      </c>
+      <c r="I71" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="72" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B72">
+        <v>4</v>
+      </c>
+      <c r="C72" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D72" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E72" t="s">
+        <v>204</v>
+      </c>
+      <c r="F72" t="s">
+        <v>157</v>
+      </c>
+      <c r="G72" t="s">
+        <v>205</v>
+      </c>
+      <c r="H72" t="s">
+        <v>139</v>
+      </c>
+      <c r="I72" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="73" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B73">
+        <v>4</v>
+      </c>
+      <c r="C73" s="2">
+        <v>46352</v>
+      </c>
+      <c r="D73" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E73" t="s">
+        <v>273</v>
+      </c>
+      <c r="F73" t="s">
+        <v>219</v>
+      </c>
+      <c r="G73" t="s">
+        <v>220</v>
+      </c>
+      <c r="H73" t="s">
+        <v>142</v>
+      </c>
+      <c r="I73" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="74" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B74">
+        <v>4</v>
+      </c>
+      <c r="C74" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="D74" s="3">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>278</v>
+      </c>
+      <c r="F74" t="s">
+        <v>151</v>
+      </c>
+      <c r="G74" t="s">
+        <v>251</v>
+      </c>
+      <c r="H74" t="s">
+        <v>208</v>
+      </c>
+      <c r="I74" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="75" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B75">
+        <v>4</v>
+      </c>
+      <c r="C75" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="D75" s="3">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>195</v>
+      </c>
+      <c r="F75" t="s">
+        <v>139</v>
+      </c>
+      <c r="G75" t="s">
+        <v>196</v>
+      </c>
+      <c r="H75" t="s">
+        <v>202</v>
+      </c>
+      <c r="I75" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="76" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B76">
+        <v>5</v>
+      </c>
+      <c r="C76" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D76" s="3">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E76" t="s">
+        <v>262</v>
+      </c>
+      <c r="F76" t="s">
+        <v>229</v>
+      </c>
+      <c r="G76" t="s">
+        <v>230</v>
+      </c>
+      <c r="H76" t="s">
+        <v>214</v>
+      </c>
+      <c r="I76" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="77" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B77">
+        <v>5</v>
+      </c>
+      <c r="C77" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D77" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E77" t="s">
+        <v>249</v>
+      </c>
+      <c r="F77" t="s">
+        <v>197</v>
+      </c>
+      <c r="G77" t="s">
+        <v>250</v>
+      </c>
+      <c r="H77" t="s">
+        <v>200</v>
+      </c>
+      <c r="I77" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="78" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B78">
+        <v>5</v>
+      </c>
+      <c r="C78" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D78" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E78" t="s">
+        <v>245</v>
+      </c>
+      <c r="F78" t="s">
+        <v>149</v>
+      </c>
+      <c r="G78" t="s">
+        <v>246</v>
+      </c>
+      <c r="H78" t="s">
+        <v>151</v>
+      </c>
+      <c r="I78" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="79" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B79">
+        <v>5</v>
+      </c>
+      <c r="C79" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D79" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E79" t="s">
+        <v>275</v>
+      </c>
+      <c r="F79" t="s">
+        <v>247</v>
+      </c>
+      <c r="G79" t="s">
+        <v>248</v>
+      </c>
+      <c r="H79" t="s">
+        <v>197</v>
+      </c>
+      <c r="I79" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="80" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B80">
+        <v>5</v>
+      </c>
+      <c r="C80" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D80" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E80" t="s">
+        <v>266</v>
+      </c>
+      <c r="F80" t="s">
+        <v>243</v>
+      </c>
+      <c r="G80" t="s">
+        <v>244</v>
+      </c>
+      <c r="H80" t="s">
+        <v>202</v>
+      </c>
+      <c r="I80" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="81" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B81">
+        <v>5</v>
+      </c>
+      <c r="C81" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D81" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E81" t="s">
+        <v>207</v>
+      </c>
+      <c r="F81" t="s">
+        <v>208</v>
+      </c>
+      <c r="G81" t="s">
+        <v>209</v>
+      </c>
+      <c r="H81" t="s">
+        <v>145</v>
+      </c>
+      <c r="I81" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="82" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B82">
+        <v>5</v>
+      </c>
+      <c r="C82" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D82" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E82" t="s">
+        <v>235</v>
+      </c>
+      <c r="F82" t="s">
+        <v>140</v>
+      </c>
+      <c r="G82" t="s">
+        <v>236</v>
+      </c>
+      <c r="H82" t="s">
+        <v>138</v>
+      </c>
+      <c r="I82" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="83" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B83">
+        <v>5</v>
+      </c>
+      <c r="C83" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D83" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E83" t="s">
+        <v>265</v>
+      </c>
+      <c r="F83" t="s">
+        <v>148</v>
+      </c>
+      <c r="G83" t="s">
+        <v>210</v>
+      </c>
+      <c r="H83" t="s">
+        <v>147</v>
+      </c>
+      <c r="I83" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="84" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B84">
+        <v>5</v>
+      </c>
+      <c r="C84" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D84" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E84" t="s">
+        <v>263</v>
+      </c>
+      <c r="F84" t="s">
+        <v>150</v>
+      </c>
+      <c r="G84" t="s">
+        <v>216</v>
+      </c>
+      <c r="H84" t="s">
+        <v>224</v>
+      </c>
+      <c r="I84" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="85" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B85">
+        <v>5</v>
+      </c>
+      <c r="C85" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D85" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="E85" t="s">
+        <v>226</v>
+      </c>
+      <c r="F85" t="s">
+        <v>227</v>
+      </c>
+      <c r="G85" t="s">
+        <v>228</v>
+      </c>
+      <c r="H85" t="s">
+        <v>142</v>
+      </c>
+      <c r="I85" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="86" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B86">
+        <v>5</v>
+      </c>
+      <c r="C86" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D86" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E86" t="s">
+        <v>252</v>
+      </c>
+      <c r="F86" t="s">
+        <v>141</v>
+      </c>
+      <c r="G86" t="s">
+        <v>253</v>
+      </c>
+      <c r="H86" t="s">
+        <v>154</v>
+      </c>
+      <c r="I86" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="87" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B87">
+        <v>5</v>
+      </c>
+      <c r="C87" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D87" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E87" t="s">
+        <v>238</v>
+      </c>
+      <c r="F87" t="s">
+        <v>146</v>
+      </c>
+      <c r="G87" t="s">
+        <v>239</v>
+      </c>
+      <c r="H87" t="s">
+        <v>219</v>
+      </c>
+      <c r="I87" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="88" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B88">
+        <v>5</v>
+      </c>
+      <c r="C88" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D88" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E88" t="s">
+        <v>274</v>
+      </c>
+      <c r="F88" t="s">
+        <v>200</v>
+      </c>
+      <c r="G88" t="s">
+        <v>261</v>
+      </c>
+      <c r="H88" t="s">
+        <v>139</v>
+      </c>
+      <c r="I88" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="89" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B89">
+        <v>5</v>
+      </c>
+      <c r="C89" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D89" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E89" t="s">
+        <v>272</v>
+      </c>
+      <c r="F89" t="s">
+        <v>197</v>
+      </c>
+      <c r="G89" t="s">
+        <v>198</v>
+      </c>
+      <c r="H89" t="s">
+        <v>153</v>
+      </c>
+      <c r="I89" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="90" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B90">
+        <v>5</v>
+      </c>
+      <c r="C90" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D90" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E90" t="s">
+        <v>231</v>
+      </c>
+      <c r="F90" t="s">
+        <v>232</v>
+      </c>
+      <c r="G90" t="s">
+        <v>233</v>
+      </c>
+      <c r="H90" t="s">
+        <v>254</v>
+      </c>
+      <c r="I90" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="91" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B91">
+        <v>5</v>
+      </c>
+      <c r="C91" s="2">
+        <v>46366</v>
+      </c>
+      <c r="D91" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E91" t="s">
+        <v>204</v>
+      </c>
+      <c r="F91" t="s">
+        <v>157</v>
+      </c>
+      <c r="G91" t="s">
+        <v>205</v>
+      </c>
+      <c r="H91" t="s">
+        <v>197</v>
+      </c>
+      <c r="I91" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="92" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B92">
+        <v>6</v>
+      </c>
+      <c r="C92" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D92" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E92" t="s">
+        <v>264</v>
+      </c>
+      <c r="F92" t="s">
+        <v>224</v>
+      </c>
+      <c r="G92" t="s">
+        <v>225</v>
+      </c>
+      <c r="H92" t="s">
+        <v>197</v>
+      </c>
+      <c r="I92" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="93" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B93">
+        <v>6</v>
+      </c>
+      <c r="C93" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D93" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E93" t="s">
+        <v>273</v>
+      </c>
+      <c r="F93" t="s">
+        <v>219</v>
+      </c>
+      <c r="G93" t="s">
+        <v>220</v>
+      </c>
+      <c r="H93" t="s">
+        <v>227</v>
+      </c>
+      <c r="I93" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="94" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B94">
+        <v>6</v>
+      </c>
+      <c r="C94" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D94" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E94" t="s">
+        <v>269</v>
+      </c>
+      <c r="F94" t="s">
+        <v>254</v>
+      </c>
+      <c r="G94" t="s">
+        <v>255</v>
+      </c>
+      <c r="H94" t="s">
+        <v>140</v>
+      </c>
+      <c r="I94" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="95" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B95">
+        <v>6</v>
+      </c>
+      <c r="C95" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D95" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E95" t="s">
+        <v>278</v>
+      </c>
+      <c r="F95" t="s">
+        <v>151</v>
+      </c>
+      <c r="G95" t="s">
+        <v>251</v>
+      </c>
+      <c r="H95" t="s">
+        <v>232</v>
+      </c>
+      <c r="I95" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="96" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B96">
+        <v>6</v>
+      </c>
+      <c r="C96" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D96" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E96" t="s">
+        <v>259</v>
+      </c>
+      <c r="F96" t="s">
+        <v>153</v>
+      </c>
+      <c r="G96" t="s">
+        <v>260</v>
+      </c>
+      <c r="H96" t="s">
+        <v>229</v>
+      </c>
+      <c r="I96" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="97" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B97">
+        <v>6</v>
+      </c>
+      <c r="C97" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D97" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E97" t="s">
+        <v>268</v>
+      </c>
+      <c r="F97" t="s">
+        <v>147</v>
+      </c>
+      <c r="G97" t="s">
+        <v>237</v>
+      </c>
+      <c r="H97" t="s">
+        <v>243</v>
+      </c>
+      <c r="I97" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="98" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B98">
+        <v>6</v>
+      </c>
+      <c r="C98" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D98" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E98" t="s">
+        <v>279</v>
+      </c>
+      <c r="F98" t="s">
+        <v>197</v>
+      </c>
+      <c r="G98" t="s">
+        <v>234</v>
+      </c>
+      <c r="H98" t="s">
+        <v>157</v>
+      </c>
+      <c r="I98" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="99" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B99">
+        <v>6</v>
+      </c>
+      <c r="C99" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D99" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E99" t="s">
+        <v>267</v>
+      </c>
+      <c r="F99" t="s">
+        <v>197</v>
+      </c>
+      <c r="G99" t="s">
+        <v>240</v>
+      </c>
+      <c r="H99" t="s">
+        <v>208</v>
+      </c>
+      <c r="I99" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="100" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B100">
+        <v>6</v>
+      </c>
+      <c r="C100" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D100" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E100" t="s">
+        <v>277</v>
+      </c>
+      <c r="F100" t="s">
+        <v>154</v>
+      </c>
+      <c r="G100" t="s">
+        <v>212</v>
+      </c>
+      <c r="H100" t="s">
+        <v>247</v>
+      </c>
+      <c r="I100" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="101" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B101">
+        <v>6</v>
+      </c>
+      <c r="C101" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D101" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E101" t="s">
+        <v>271</v>
+      </c>
+      <c r="F101" t="s">
+        <v>136</v>
+      </c>
+      <c r="G101" t="s">
+        <v>258</v>
+      </c>
+      <c r="H101" t="s">
+        <v>146</v>
+      </c>
+      <c r="I101" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="102" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B102">
+        <v>6</v>
+      </c>
+      <c r="C102" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D102" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E102" t="s">
+        <v>270</v>
+      </c>
+      <c r="F102" t="s">
+        <v>202</v>
+      </c>
+      <c r="G102" t="s">
+        <v>203</v>
+      </c>
+      <c r="H102" t="s">
+        <v>148</v>
+      </c>
+      <c r="I102" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="103" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B103">
+        <v>6</v>
+      </c>
+      <c r="C103" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D103" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E103" t="s">
+        <v>217</v>
+      </c>
+      <c r="F103" t="s">
+        <v>138</v>
+      </c>
+      <c r="G103" t="s">
+        <v>218</v>
+      </c>
+      <c r="H103" t="s">
+        <v>141</v>
+      </c>
+      <c r="I103" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="104" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B104">
+        <v>6</v>
+      </c>
+      <c r="C104" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D104" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E104" t="s">
+        <v>256</v>
+      </c>
+      <c r="F104" t="s">
+        <v>142</v>
+      </c>
+      <c r="G104" t="s">
+        <v>257</v>
+      </c>
+      <c r="H104" t="s">
+        <v>222</v>
+      </c>
+      <c r="I104" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="105" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B105">
+        <v>6</v>
+      </c>
+      <c r="C105" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D105" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E105" t="s">
+        <v>276</v>
+      </c>
+      <c r="F105" t="s">
+        <v>153</v>
+      </c>
+      <c r="G105" t="s">
+        <v>206</v>
+      </c>
+      <c r="H105" t="s">
+        <v>150</v>
+      </c>
+      <c r="I105" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="106" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B106">
+        <v>6</v>
+      </c>
+      <c r="C106" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D106" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E106" t="s">
+        <v>107</v>
+      </c>
+      <c r="F106" t="s">
+        <v>145</v>
+      </c>
+      <c r="G106" t="s">
+        <v>211</v>
+      </c>
+      <c r="H106" t="s">
+        <v>200</v>
+      </c>
+      <c r="I106" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="107" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B107">
+        <v>6</v>
+      </c>
+      <c r="C107" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D107" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E107" t="s">
+        <v>199</v>
+      </c>
+      <c r="F107" t="s">
+        <v>200</v>
+      </c>
+      <c r="G107" t="s">
+        <v>201</v>
+      </c>
+      <c r="H107" t="s">
+        <v>139</v>
+      </c>
+      <c r="I107" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="108" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B108">
+        <v>6</v>
+      </c>
+      <c r="C108" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D108" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E108" t="s">
+        <v>213</v>
+      </c>
+      <c r="F108" t="s">
+        <v>214</v>
+      </c>
+      <c r="G108" t="s">
+        <v>215</v>
+      </c>
+      <c r="H108" t="s">
+        <v>197</v>
+      </c>
+      <c r="I108" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="109" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B109">
+        <v>6</v>
+      </c>
+      <c r="C109" s="2">
+        <v>46373</v>
+      </c>
+      <c r="D109" s="3">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E109" t="s">
+        <v>195</v>
+      </c>
+      <c r="F109" t="s">
+        <v>139</v>
+      </c>
+      <c r="G109" t="s">
+        <v>196</v>
+      </c>
+      <c r="H109" t="s">
+        <v>149</v>
+      </c>
+      <c r="I109" t="s">
+        <v>246</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>